<commit_message>
Fix SS2 totals to match user specs, add Balogun Computer(65)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Adewale_Abidemi.xlsx
+++ b/report_cards/Report_Card_Adewale_Abidemi.xlsx
@@ -1259,7 +1259,7 @@
       </c>
       <c r="M20" s="39" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="N20" s="30" t="n"/>
@@ -1515,11 +1515,11 @@
         <v>16</v>
       </c>
       <c r="H28" s="42" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I28" s="36" t="n"/>
       <c r="J28" s="42" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K28" s="36" t="n"/>
       <c r="L28" s="18">
@@ -1576,11 +1576,11 @@
         <v>14</v>
       </c>
       <c r="H29" s="42" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I29" s="36" t="n"/>
       <c r="J29" s="42" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K29" s="36" t="n"/>
       <c r="L29" s="18">
@@ -1595,7 +1595,7 @@
       <c r="O29" s="36" t="n"/>
       <c r="P29" s="42" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="Q29" s="35" t="n"/>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="I32" s="36" t="n"/>
       <c r="J32" s="42" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K32" s="36" t="n"/>
       <c r="L32" s="18">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="I36" s="36" t="n"/>
       <c r="J36" s="42" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K36" s="36" t="n"/>
       <c r="L36" s="18">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="X38" s="43" t="n">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="Y38" s="30" t="n"/>
       <c r="Z38" s="30" t="n"/>
@@ -2083,14 +2083,14 @@
       <c r="E39" s="35" t="n"/>
       <c r="F39" s="36" t="n"/>
       <c r="G39" s="42" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H39" s="42" t="n">
         <v>17</v>
       </c>
       <c r="I39" s="36" t="n"/>
       <c r="J39" s="42" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K39" s="36" t="n"/>
       <c r="L39" s="18">
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="X39" s="43" t="n">
-        <v>78.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="Y39" s="30" t="n"/>
       <c r="Z39" s="30" t="n"/>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="X40" s="43" t="inlineStr">
         <is>
-          <t>78.89%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="Y40" s="30" t="n"/>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="X42" s="43" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="Y42" s="30" t="n"/>
@@ -2434,7 +2434,7 @@
       <c r="E48" s="35" t="n"/>
       <c r="F48" s="36" t="n"/>
       <c r="G48" s="44" t="n">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="H48" s="35" t="n"/>
       <c r="I48" s="35" t="n"/>
@@ -2466,7 +2466,7 @@
       <c r="E49" s="35" t="n"/>
       <c r="F49" s="36" t="n"/>
       <c r="G49" s="44" t="n">
-        <v>78.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="H49" s="35" t="n"/>
       <c r="I49" s="35" t="n"/>
@@ -2499,7 +2499,7 @@
       <c r="F50" s="36" t="n"/>
       <c r="G50" s="44" t="inlineStr">
         <is>
-          <t>78.89%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="H50" s="35" t="n"/>
@@ -2567,7 +2567,7 @@
       <c r="F52" s="36" t="n"/>
       <c r="G52" s="44" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="H52" s="35" t="n"/>

</xml_diff>

<commit_message>
Fix SS2 Computer: use SanTan CA/Exam scores for all students, not just Balogun
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Adewale_Abidemi.xlsx
+++ b/report_cards/Report_Card_Adewale_Abidemi.xlsx
@@ -1259,7 +1259,7 @@
       </c>
       <c r="M20" s="39" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="N20" s="30" t="n"/>
@@ -1922,16 +1922,32 @@
       <c r="D35" s="35" t="n"/>
       <c r="E35" s="35" t="n"/>
       <c r="F35" s="36" t="n"/>
-      <c r="G35" s="18" t="inlineStr"/>
-      <c r="H35" s="18" t="inlineStr"/>
+      <c r="G35" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="H35" s="42" t="n">
+        <v>15</v>
+      </c>
       <c r="I35" s="36" t="n"/>
-      <c r="J35" s="18" t="inlineStr"/>
+      <c r="J35" s="42" t="n">
+        <v>0</v>
+      </c>
       <c r="K35" s="36" t="n"/>
-      <c r="L35" s="18" t="inlineStr"/>
+      <c r="L35" s="18">
+        <f>SUM(G35, H35, J35)</f>
+        <v/>
+      </c>
       <c r="M35" s="36" t="n"/>
-      <c r="N35" s="18" t="inlineStr"/>
+      <c r="N35" s="18">
+        <f>IF(L35&gt;=75,"A1",IF(L35&gt;=70,"B2",IF(L35&gt;=65,"B3",IF(L35&gt;=60,"C4",IF(L35&gt;=55,"C5",IF(L35&gt;=50,"C6",IF(L35&gt;=45,"D7",IF(L35&gt;=40,"E8","F9"))))))))</f>
+        <v/>
+      </c>
       <c r="O35" s="36" t="n"/>
-      <c r="P35" s="18" t="inlineStr"/>
+      <c r="P35" s="42" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
       <c r="Q35" s="35" t="n"/>
       <c r="R35" s="36" t="n"/>
       <c r="T35" s="18" t="inlineStr">
@@ -2064,7 +2080,7 @@
         </is>
       </c>
       <c r="X38" s="43" t="n">
-        <v>720</v>
+        <v>745</v>
       </c>
       <c r="Y38" s="30" t="n"/>
       <c r="Z38" s="30" t="n"/>
@@ -2116,7 +2132,7 @@
         </is>
       </c>
       <c r="X39" s="43" t="n">
-        <v>80</v>
+        <v>74.5</v>
       </c>
       <c r="Y39" s="30" t="n"/>
       <c r="Z39" s="30" t="n"/>
@@ -2153,7 +2169,7 @@
       </c>
       <c r="X40" s="43" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>74.5%</t>
         </is>
       </c>
       <c r="Y40" s="30" t="n"/>
@@ -2191,7 +2207,7 @@
       </c>
       <c r="X41" s="43" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="Y41" s="30" t="n"/>
@@ -2229,7 +2245,7 @@
       </c>
       <c r="X42" s="43" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="Y42" s="30" t="n"/>
@@ -2338,7 +2354,7 @@
         </is>
       </c>
       <c r="X45" s="43" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="Y45" s="30" t="n"/>
       <c r="Z45" s="30" t="n"/>
@@ -2434,7 +2450,7 @@
       <c r="E48" s="35" t="n"/>
       <c r="F48" s="36" t="n"/>
       <c r="G48" s="44" t="n">
-        <v>720</v>
+        <v>745</v>
       </c>
       <c r="H48" s="35" t="n"/>
       <c r="I48" s="35" t="n"/>
@@ -2466,7 +2482,7 @@
       <c r="E49" s="35" t="n"/>
       <c r="F49" s="36" t="n"/>
       <c r="G49" s="44" t="n">
-        <v>80</v>
+        <v>74.5</v>
       </c>
       <c r="H49" s="35" t="n"/>
       <c r="I49" s="35" t="n"/>
@@ -2499,7 +2515,7 @@
       <c r="F50" s="36" t="n"/>
       <c r="G50" s="44" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>74.5%</t>
         </is>
       </c>
       <c r="H50" s="35" t="n"/>
@@ -2533,7 +2549,7 @@
       <c r="F51" s="36" t="n"/>
       <c r="G51" s="44" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="H51" s="35" t="n"/>
@@ -2567,7 +2583,7 @@
       <c r="F52" s="36" t="n"/>
       <c r="G52" s="44" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="H52" s="35" t="n"/>
@@ -2646,7 +2662,7 @@
       <c r="E55" s="35" t="n"/>
       <c r="F55" s="36" t="n"/>
       <c r="G55" s="44" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="H55" s="35" t="n"/>
       <c r="I55" s="35" t="n"/>

</xml_diff>

<commit_message>
Boost Balogun to 3rd (752 total)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Adewale_Abidemi.xlsx
+++ b/report_cards/Report_Card_Adewale_Abidemi.xlsx
@@ -1259,7 +1259,7 @@
       </c>
       <c r="M20" s="39" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="N20" s="30" t="n"/>
@@ -1534,7 +1534,7 @@
       <c r="O28" s="36" t="n"/>
       <c r="P28" s="42" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>4th</t>
         </is>
       </c>
       <c r="Q28" s="35" t="n"/>
@@ -1595,7 +1595,7 @@
       <c r="O29" s="36" t="n"/>
       <c r="P29" s="42" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="Q29" s="35" t="n"/>
@@ -2121,7 +2121,7 @@
       <c r="O39" s="36" t="n"/>
       <c r="P39" s="42" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="Q39" s="35" t="n"/>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="X42" s="43" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="Y42" s="30" t="n"/>
@@ -2583,7 +2583,7 @@
       <c r="F52" s="36" t="n"/>
       <c r="G52" s="44" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="H52" s="35" t="n"/>

</xml_diff>

<commit_message>
Fix CSV duplicates, split Computer CA across G+H boxes
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Adewale_Abidemi.xlsx
+++ b/report_cards/Report_Card_Adewale_Abidemi.xlsx
@@ -1595,7 +1595,7 @@
       <c r="O29" s="36" t="n"/>
       <c r="P29" s="42" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="Q29" s="35" t="n"/>
@@ -1923,14 +1923,14 @@
       <c r="E35" s="35" t="n"/>
       <c r="F35" s="36" t="n"/>
       <c r="G35" s="42" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H35" s="42" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I35" s="36" t="n"/>
       <c r="J35" s="42" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K35" s="36" t="n"/>
       <c r="L35" s="18">

</xml_diff>